<commit_message>
chore(data-release): publish site data 2026-09-27 02:03:57 UTC
</commit_message>
<xml_diff>
--- a/countries/at/2020-2025.xlsx
+++ b/countries/at/2020-2025.xlsx
@@ -75008,17 +75008,17 @@
       </c>
       <c r="H380" t="inlineStr">
         <is>
-          <t>D017</t>
+          <t>D007</t>
         </is>
       </c>
       <c r="I380" t="inlineStr">
         <is>
-          <t>Measles</t>
+          <t>Hepatitis A</t>
         </is>
       </c>
       <c r="J380" t="inlineStr">
         <is>
-          <t>麻疹</t>
+          <t>甲型肝炎</t>
         </is>
       </c>
       <c r="K380" t="inlineStr">
@@ -75037,13 +75037,13 @@
         </is>
       </c>
       <c r="N380" t="n">
-        <v>152</v>
+        <v>248</v>
       </c>
       <c r="O380" t="n">
-        <v>152</v>
+        <v>248</v>
       </c>
       <c r="R380" t="n">
-        <v>1.667841836802993</v>
+        <v>2.721215628468041</v>
       </c>
       <c r="S380" t="inlineStr">
         <is>
@@ -75052,7 +75052,7 @@
       </c>
       <c r="U380" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_MEAS_ANNUAL</t>
+          <t>SER_AT_ECDC_HEPA_ANNUAL</t>
         </is>
       </c>
       <c r="AA380" t="inlineStr">
@@ -75077,7 +75077,7 @@
       </c>
       <c r="AS380" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_MEAS_ANNUAL</t>
+          <t>SER_AT_ECDC_HEPA_ANNUAL</t>
         </is>
       </c>
       <c r="AT380" t="n">
@@ -75167,17 +75167,17 @@
       </c>
       <c r="H381" t="inlineStr">
         <is>
-          <t>D017</t>
+          <t>D007</t>
         </is>
       </c>
       <c r="I381" t="inlineStr">
         <is>
-          <t>Measles</t>
+          <t>Hepatitis A</t>
         </is>
       </c>
       <c r="J381" t="inlineStr">
         <is>
-          <t>麻疹</t>
+          <t>甲型肝炎</t>
         </is>
       </c>
       <c r="K381" t="inlineStr">
@@ -75196,19 +75196,19 @@
         </is>
       </c>
       <c r="N381" t="n">
-        <v>152</v>
+        <v>248</v>
       </c>
       <c r="O381" t="n">
-        <v>152</v>
+        <v>248</v>
       </c>
       <c r="U381" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_MEAS_ANNUAL</t>
+          <t>SER_AT_ECDC_HEPA_ANNUAL</t>
         </is>
       </c>
       <c r="V381" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_MEAS_ANNUAL</t>
+          <t>SER_AT_ECDC_HEPA_ANNUAL</t>
         </is>
       </c>
       <c r="W381" t="inlineStr">
@@ -75218,7 +75218,7 @@
       </c>
       <c r="X381" t="inlineStr">
         <is>
-          <t>Measles</t>
+          <t>Hepatitis A</t>
         </is>
       </c>
       <c r="Y381" t="inlineStr">
@@ -75311,7 +75311,7 @@
       </c>
       <c r="AS381" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_MEAS_ANNUAL</t>
+          <t>SER_AT_ECDC_HEPA_ANNUAL</t>
         </is>
       </c>
       <c r="AT381" t="n">
@@ -75401,22 +75401,22 @@
       </c>
       <c r="H382" t="inlineStr">
         <is>
-          <t>D029</t>
+          <t>D017</t>
         </is>
       </c>
       <c r="I382" t="inlineStr">
         <is>
-          <t>Diphtheria</t>
+          <t>Measles</t>
         </is>
       </c>
       <c r="J382" t="inlineStr">
         <is>
-          <t>白喉</t>
+          <t>麻疹</t>
         </is>
       </c>
       <c r="K382" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L382" t="inlineStr">
@@ -75430,13 +75430,13 @@
         </is>
       </c>
       <c r="N382" t="n">
-        <v>3</v>
+        <v>152</v>
       </c>
       <c r="O382" t="n">
-        <v>3</v>
+        <v>152</v>
       </c>
       <c r="R382" t="n">
-        <v>0.03291793098953275</v>
+        <v>1.667841836802993</v>
       </c>
       <c r="S382" t="inlineStr">
         <is>
@@ -75445,7 +75445,7 @@
       </c>
       <c r="U382" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_DIPH_ANNUAL</t>
+          <t>SER_AT_ECDC_MEAS_ANNUAL</t>
         </is>
       </c>
       <c r="AA382" t="inlineStr">
@@ -75470,7 +75470,7 @@
       </c>
       <c r="AS382" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_DIPH_ANNUAL</t>
+          <t>SER_AT_ECDC_MEAS_ANNUAL</t>
         </is>
       </c>
       <c r="AT382" t="n">
@@ -75560,22 +75560,22 @@
       </c>
       <c r="H383" t="inlineStr">
         <is>
-          <t>D029</t>
+          <t>D017</t>
         </is>
       </c>
       <c r="I383" t="inlineStr">
         <is>
-          <t>Diphtheria</t>
+          <t>Measles</t>
         </is>
       </c>
       <c r="J383" t="inlineStr">
         <is>
-          <t>白喉</t>
+          <t>麻疹</t>
         </is>
       </c>
       <c r="K383" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L383" t="inlineStr">
@@ -75589,19 +75589,19 @@
         </is>
       </c>
       <c r="N383" t="n">
-        <v>3</v>
+        <v>152</v>
       </c>
       <c r="O383" t="n">
-        <v>3</v>
+        <v>152</v>
       </c>
       <c r="U383" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_DIPH_ANNUAL</t>
+          <t>SER_AT_ECDC_MEAS_ANNUAL</t>
         </is>
       </c>
       <c r="V383" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_DIPH_ANNUAL</t>
+          <t>SER_AT_ECDC_MEAS_ANNUAL</t>
         </is>
       </c>
       <c r="W383" t="inlineStr">
@@ -75611,7 +75611,7 @@
       </c>
       <c r="X383" t="inlineStr">
         <is>
-          <t>Diphtheria</t>
+          <t>Measles</t>
         </is>
       </c>
       <c r="Y383" t="inlineStr">
@@ -75704,7 +75704,7 @@
       </c>
       <c r="AS383" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_DIPH_ANNUAL</t>
+          <t>SER_AT_ECDC_MEAS_ANNUAL</t>
         </is>
       </c>
       <c r="AT383" t="n">
@@ -75794,22 +75794,22 @@
       </c>
       <c r="H384" t="inlineStr">
         <is>
-          <t>D040</t>
+          <t>D029</t>
         </is>
       </c>
       <c r="I384" t="inlineStr">
         <is>
-          <t>Rubella</t>
+          <t>Diphtheria</t>
         </is>
       </c>
       <c r="J384" t="inlineStr">
         <is>
-          <t>风疹</t>
+          <t>白喉</t>
         </is>
       </c>
       <c r="K384" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L384" t="inlineStr">
@@ -75823,13 +75823,13 @@
         </is>
       </c>
       <c r="N384" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O384" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R384" t="n">
-        <v>0</v>
+        <v>0.03291793098953275</v>
       </c>
       <c r="S384" t="inlineStr">
         <is>
@@ -75838,7 +75838,7 @@
       </c>
       <c r="U384" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_RUBE_ANNUAL</t>
+          <t>SER_AT_ECDC_DIPH_ANNUAL</t>
         </is>
       </c>
       <c r="AA384" t="inlineStr">
@@ -75863,7 +75863,7 @@
       </c>
       <c r="AS384" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_RUBE_ANNUAL</t>
+          <t>SER_AT_ECDC_DIPH_ANNUAL</t>
         </is>
       </c>
       <c r="AT384" t="n">
@@ -75953,22 +75953,22 @@
       </c>
       <c r="H385" t="inlineStr">
         <is>
-          <t>D040</t>
+          <t>D029</t>
         </is>
       </c>
       <c r="I385" t="inlineStr">
         <is>
-          <t>Rubella</t>
+          <t>Diphtheria</t>
         </is>
       </c>
       <c r="J385" t="inlineStr">
         <is>
-          <t>风疹</t>
+          <t>白喉</t>
         </is>
       </c>
       <c r="K385" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L385" t="inlineStr">
@@ -75982,19 +75982,19 @@
         </is>
       </c>
       <c r="N385" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O385" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="U385" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_RUBE_ANNUAL</t>
+          <t>SER_AT_ECDC_DIPH_ANNUAL</t>
         </is>
       </c>
       <c r="V385" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_RUBE_ANNUAL</t>
+          <t>SER_AT_ECDC_DIPH_ANNUAL</t>
         </is>
       </c>
       <c r="W385" t="inlineStr">
@@ -76004,7 +76004,7 @@
       </c>
       <c r="X385" t="inlineStr">
         <is>
-          <t>Rubella</t>
+          <t>Diphtheria</t>
         </is>
       </c>
       <c r="Y385" t="inlineStr">
@@ -76097,7 +76097,7 @@
       </c>
       <c r="AS385" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_RUBE_ANNUAL</t>
+          <t>SER_AT_ECDC_DIPH_ANNUAL</t>
         </is>
       </c>
       <c r="AT385" t="n">
@@ -76187,17 +76187,17 @@
       </c>
       <c r="H386" t="inlineStr">
         <is>
-          <t>D107</t>
+          <t>D032</t>
         </is>
       </c>
       <c r="I386" t="inlineStr">
         <is>
-          <t>Legionellosis</t>
+          <t>Brucellosis</t>
         </is>
       </c>
       <c r="J386" t="inlineStr">
         <is>
-          <t>军团菌病</t>
+          <t>布鲁氏菌病</t>
         </is>
       </c>
       <c r="K386" t="inlineStr">
@@ -76216,13 +76216,13 @@
         </is>
       </c>
       <c r="N386" t="n">
-        <v>419</v>
+        <v>8</v>
       </c>
       <c r="O386" t="n">
-        <v>419</v>
+        <v>8</v>
       </c>
       <c r="R386" t="n">
-        <v>4.597537694871408</v>
+        <v>0.08778114930542068</v>
       </c>
       <c r="S386" t="inlineStr">
         <is>
@@ -76231,7 +76231,7 @@
       </c>
       <c r="U386" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_LEGI_ANNUAL</t>
+          <t>SER_AT_ECDC_BRUC_ANNUAL</t>
         </is>
       </c>
       <c r="AA386" t="inlineStr">
@@ -76256,7 +76256,7 @@
       </c>
       <c r="AS386" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_LEGI_ANNUAL</t>
+          <t>SER_AT_ECDC_BRUC_ANNUAL</t>
         </is>
       </c>
       <c r="AT386" t="n">
@@ -76346,17 +76346,17 @@
       </c>
       <c r="H387" t="inlineStr">
         <is>
-          <t>D107</t>
+          <t>D032</t>
         </is>
       </c>
       <c r="I387" t="inlineStr">
         <is>
-          <t>Legionellosis</t>
+          <t>Brucellosis</t>
         </is>
       </c>
       <c r="J387" t="inlineStr">
         <is>
-          <t>军团菌病</t>
+          <t>布鲁氏菌病</t>
         </is>
       </c>
       <c r="K387" t="inlineStr">
@@ -76375,19 +76375,19 @@
         </is>
       </c>
       <c r="N387" t="n">
-        <v>419</v>
+        <v>8</v>
       </c>
       <c r="O387" t="n">
-        <v>419</v>
+        <v>8</v>
       </c>
       <c r="U387" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_LEGI_ANNUAL</t>
+          <t>SER_AT_ECDC_BRUC_ANNUAL</t>
         </is>
       </c>
       <c r="V387" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_LEGI_ANNUAL</t>
+          <t>SER_AT_ECDC_BRUC_ANNUAL</t>
         </is>
       </c>
       <c r="W387" t="inlineStr">
@@ -76397,7 +76397,7 @@
       </c>
       <c r="X387" t="inlineStr">
         <is>
-          <t>Legionnaires' disease</t>
+          <t>Brucellosis</t>
         </is>
       </c>
       <c r="Y387" t="inlineStr">
@@ -76490,7 +76490,7 @@
       </c>
       <c r="AS387" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_LEGI_ANNUAL</t>
+          <t>SER_AT_ECDC_BRUC_ANNUAL</t>
         </is>
       </c>
       <c r="AT387" t="n">
@@ -76537,6 +76537,3543 @@
         </is>
       </c>
       <c r="BC387" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t>D040</t>
+        </is>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>Rubella</t>
+        </is>
+      </c>
+      <c r="J388" t="inlineStr">
+        <is>
+          <t>风疹</t>
+        </is>
+      </c>
+      <c r="K388" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L388" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M388" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N388" t="n">
+        <v>0</v>
+      </c>
+      <c r="O388" t="n">
+        <v>0</v>
+      </c>
+      <c r="R388" t="n">
+        <v>0</v>
+      </c>
+      <c r="S388" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U388" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_RUBE_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA388" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO388" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP388" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ388" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS388" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_RUBE_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT388" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU388" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV388" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW388" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX388" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY388" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ388" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA388" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB388" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC388" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t>D040</t>
+        </is>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>Rubella</t>
+        </is>
+      </c>
+      <c r="J389" t="inlineStr">
+        <is>
+          <t>风疹</t>
+        </is>
+      </c>
+      <c r="K389" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L389" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M389" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N389" t="n">
+        <v>0</v>
+      </c>
+      <c r="O389" t="n">
+        <v>0</v>
+      </c>
+      <c r="U389" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_RUBE_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V389" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_RUBE_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W389" t="inlineStr">
+        <is>
+          <t>SRC_AT_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X389" t="inlineStr">
+        <is>
+          <t>Rubella</t>
+        </is>
+      </c>
+      <c r="Y389" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z389" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA389" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB389" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC389" t="inlineStr">
+        <is>
+          <t>country:AT:national</t>
+        </is>
+      </c>
+      <c r="AD389" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE389" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF389" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG389" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH389" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI389" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ389" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK389" t="inlineStr">
+        <is>
+          <t>Austria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM389" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN389" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO389" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP389" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ389" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS389" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_RUBE_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT389" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU389" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV389" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW389" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX389" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY389" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ389" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA389" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB389" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC389" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>D045</t>
+        </is>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>Echinococcosis</t>
+        </is>
+      </c>
+      <c r="J390" t="inlineStr">
+        <is>
+          <t>包虫病</t>
+        </is>
+      </c>
+      <c r="K390" t="inlineStr">
+        <is>
+          <t>Parasitic</t>
+        </is>
+      </c>
+      <c r="L390" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M390" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N390" t="n">
+        <v>47</v>
+      </c>
+      <c r="O390" t="n">
+        <v>47</v>
+      </c>
+      <c r="R390" t="n">
+        <v>0.5157142521693465</v>
+      </c>
+      <c r="S390" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U390" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_ECHI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA390" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO390" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP390" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ390" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS390" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_ECHI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT390" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU390" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV390" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW390" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX390" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY390" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ390" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA390" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB390" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC390" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>D045</t>
+        </is>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>Echinococcosis</t>
+        </is>
+      </c>
+      <c r="J391" t="inlineStr">
+        <is>
+          <t>包虫病</t>
+        </is>
+      </c>
+      <c r="K391" t="inlineStr">
+        <is>
+          <t>Parasitic</t>
+        </is>
+      </c>
+      <c r="L391" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M391" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N391" t="n">
+        <v>47</v>
+      </c>
+      <c r="O391" t="n">
+        <v>47</v>
+      </c>
+      <c r="U391" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_ECHI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V391" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_ECHI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W391" t="inlineStr">
+        <is>
+          <t>SRC_AT_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X391" t="inlineStr">
+        <is>
+          <t>Echinococcosis</t>
+        </is>
+      </c>
+      <c r="Y391" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z391" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA391" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB391" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC391" t="inlineStr">
+        <is>
+          <t>country:AT:national</t>
+        </is>
+      </c>
+      <c r="AD391" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE391" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF391" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG391" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH391" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI391" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ391" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK391" t="inlineStr">
+        <is>
+          <t>Austria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM391" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN391" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO391" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP391" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ391" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS391" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_ECHI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT391" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU391" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV391" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW391" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX391" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY391" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ391" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA391" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB391" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC391" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>D092</t>
+        </is>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>Campylobacteriosis</t>
+        </is>
+      </c>
+      <c r="J392" t="inlineStr">
+        <is>
+          <t>弯曲杆菌病</t>
+        </is>
+      </c>
+      <c r="K392" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L392" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M392" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N392" t="n">
+        <v>7151</v>
+      </c>
+      <c r="O392" t="n">
+        <v>7151</v>
+      </c>
+      <c r="R392" t="n">
+        <v>78.46537483538292</v>
+      </c>
+      <c r="S392" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U392" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_CAMP_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA392" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO392" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP392" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ392" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS392" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_CAMP_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT392" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU392" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV392" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW392" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX392" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY392" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ392" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA392" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB392" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC392" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>D092</t>
+        </is>
+      </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>Campylobacteriosis</t>
+        </is>
+      </c>
+      <c r="J393" t="inlineStr">
+        <is>
+          <t>弯曲杆菌病</t>
+        </is>
+      </c>
+      <c r="K393" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L393" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M393" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N393" t="n">
+        <v>7151</v>
+      </c>
+      <c r="O393" t="n">
+        <v>7151</v>
+      </c>
+      <c r="U393" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_CAMP_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V393" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_CAMP_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W393" t="inlineStr">
+        <is>
+          <t>SRC_AT_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X393" t="inlineStr">
+        <is>
+          <t>Campylobacteriosis</t>
+        </is>
+      </c>
+      <c r="Y393" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z393" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA393" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB393" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC393" t="inlineStr">
+        <is>
+          <t>country:AT:national</t>
+        </is>
+      </c>
+      <c r="AD393" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE393" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF393" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG393" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH393" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI393" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ393" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK393" t="inlineStr">
+        <is>
+          <t>Austria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM393" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN393" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO393" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP393" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ393" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS393" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_CAMP_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT393" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU393" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV393" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW393" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX393" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY393" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ393" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA393" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB393" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC393" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>D105</t>
+        </is>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>Shigellosis</t>
+        </is>
+      </c>
+      <c r="J394" t="inlineStr">
+        <is>
+          <t>志贺菌病</t>
+        </is>
+      </c>
+      <c r="K394" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L394" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M394" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N394" t="n">
+        <v>98</v>
+      </c>
+      <c r="O394" t="n">
+        <v>98</v>
+      </c>
+      <c r="R394" t="n">
+        <v>1.075319078991403</v>
+      </c>
+      <c r="S394" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U394" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_SHIG_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA394" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO394" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP394" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ394" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS394" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_SHIG_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT394" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU394" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV394" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW394" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX394" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY394" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ394" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA394" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB394" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC394" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>D105</t>
+        </is>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>Shigellosis</t>
+        </is>
+      </c>
+      <c r="J395" t="inlineStr">
+        <is>
+          <t>志贺菌病</t>
+        </is>
+      </c>
+      <c r="K395" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L395" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M395" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N395" t="n">
+        <v>98</v>
+      </c>
+      <c r="O395" t="n">
+        <v>98</v>
+      </c>
+      <c r="U395" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_SHIG_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V395" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_SHIG_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W395" t="inlineStr">
+        <is>
+          <t>SRC_AT_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X395" t="inlineStr">
+        <is>
+          <t>Shigellosis</t>
+        </is>
+      </c>
+      <c r="Y395" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z395" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA395" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB395" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC395" t="inlineStr">
+        <is>
+          <t>country:AT:national</t>
+        </is>
+      </c>
+      <c r="AD395" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE395" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF395" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG395" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH395" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI395" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ395" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK395" t="inlineStr">
+        <is>
+          <t>Austria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM395" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN395" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO395" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP395" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ395" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS395" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_SHIG_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT395" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU395" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV395" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW395" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX395" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY395" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ395" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA395" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB395" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC395" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>D107</t>
+        </is>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>Legionellosis</t>
+        </is>
+      </c>
+      <c r="J396" t="inlineStr">
+        <is>
+          <t>军团菌病</t>
+        </is>
+      </c>
+      <c r="K396" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L396" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M396" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N396" t="n">
+        <v>419</v>
+      </c>
+      <c r="O396" t="n">
+        <v>419</v>
+      </c>
+      <c r="R396" t="n">
+        <v>4.597537694871408</v>
+      </c>
+      <c r="S396" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U396" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_LEGI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA396" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO396" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP396" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ396" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS396" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_LEGI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT396" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU396" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV396" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW396" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX396" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY396" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ396" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA396" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB396" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC396" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t>D107</t>
+        </is>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>Legionellosis</t>
+        </is>
+      </c>
+      <c r="J397" t="inlineStr">
+        <is>
+          <t>军团菌病</t>
+        </is>
+      </c>
+      <c r="K397" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L397" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M397" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N397" t="n">
+        <v>419</v>
+      </c>
+      <c r="O397" t="n">
+        <v>419</v>
+      </c>
+      <c r="U397" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_LEGI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V397" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_LEGI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W397" t="inlineStr">
+        <is>
+          <t>SRC_AT_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X397" t="inlineStr">
+        <is>
+          <t>Legionnaires' disease</t>
+        </is>
+      </c>
+      <c r="Y397" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z397" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA397" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB397" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC397" t="inlineStr">
+        <is>
+          <t>country:AT:national</t>
+        </is>
+      </c>
+      <c r="AD397" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE397" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF397" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG397" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH397" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI397" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ397" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK397" t="inlineStr">
+        <is>
+          <t>Austria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM397" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN397" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO397" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP397" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ397" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS397" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_LEGI_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT397" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU397" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV397" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW397" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX397" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY397" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ397" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA397" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB397" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC397" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H398" t="inlineStr">
+        <is>
+          <t>D108</t>
+        </is>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>Listeriosis</t>
+        </is>
+      </c>
+      <c r="J398" t="inlineStr">
+        <is>
+          <t>李斯特菌病</t>
+        </is>
+      </c>
+      <c r="K398" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L398" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M398" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N398" t="n">
+        <v>32</v>
+      </c>
+      <c r="O398" t="n">
+        <v>32</v>
+      </c>
+      <c r="R398" t="n">
+        <v>0.3511245972216827</v>
+      </c>
+      <c r="S398" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U398" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_LIST_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA398" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO398" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP398" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ398" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS398" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_LIST_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT398" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU398" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV398" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW398" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX398" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY398" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ398" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA398" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB398" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC398" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H399" t="inlineStr">
+        <is>
+          <t>D108</t>
+        </is>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>Listeriosis</t>
+        </is>
+      </c>
+      <c r="J399" t="inlineStr">
+        <is>
+          <t>李斯特菌病</t>
+        </is>
+      </c>
+      <c r="K399" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L399" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M399" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N399" t="n">
+        <v>32</v>
+      </c>
+      <c r="O399" t="n">
+        <v>32</v>
+      </c>
+      <c r="U399" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_LIST_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V399" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_LIST_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W399" t="inlineStr">
+        <is>
+          <t>SRC_AT_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X399" t="inlineStr">
+        <is>
+          <t>Listeriosis</t>
+        </is>
+      </c>
+      <c r="Y399" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z399" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA399" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB399" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC399" t="inlineStr">
+        <is>
+          <t>country:AT:national</t>
+        </is>
+      </c>
+      <c r="AD399" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE399" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF399" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG399" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH399" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI399" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ399" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK399" t="inlineStr">
+        <is>
+          <t>Austria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM399" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN399" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO399" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP399" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ399" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS399" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_LIST_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT399" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU399" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV399" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW399" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX399" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY399" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ399" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA399" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB399" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC399" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t>D114</t>
+        </is>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>Salmonellosis</t>
+        </is>
+      </c>
+      <c r="J400" t="inlineStr">
+        <is>
+          <t>沙门氏菌病</t>
+        </is>
+      </c>
+      <c r="K400" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L400" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M400" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N400" t="n">
+        <v>1528</v>
+      </c>
+      <c r="O400" t="n">
+        <v>1528</v>
+      </c>
+      <c r="R400" t="n">
+        <v>16.76619951733535</v>
+      </c>
+      <c r="S400" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U400" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_SALM_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA400" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO400" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP400" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ400" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS400" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_SALM_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT400" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU400" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV400" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW400" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX400" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY400" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ400" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA400" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB400" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC400" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t>D114</t>
+        </is>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>Salmonellosis</t>
+        </is>
+      </c>
+      <c r="J401" t="inlineStr">
+        <is>
+          <t>沙门氏菌病</t>
+        </is>
+      </c>
+      <c r="K401" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L401" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M401" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N401" t="n">
+        <v>1528</v>
+      </c>
+      <c r="O401" t="n">
+        <v>1528</v>
+      </c>
+      <c r="U401" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_SALM_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V401" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_SALM_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W401" t="inlineStr">
+        <is>
+          <t>SRC_AT_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X401" t="inlineStr">
+        <is>
+          <t>Salmonellosis</t>
+        </is>
+      </c>
+      <c r="Y401" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z401" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA401" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB401" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC401" t="inlineStr">
+        <is>
+          <t>country:AT:national</t>
+        </is>
+      </c>
+      <c r="AD401" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE401" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF401" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG401" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH401" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI401" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ401" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK401" t="inlineStr">
+        <is>
+          <t>Austria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM401" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN401" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO401" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP401" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ401" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS401" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_SALM_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT401" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU401" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV401" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW401" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX401" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY401" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ401" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA401" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB401" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC401" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>D115</t>
+        </is>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>Shiga toxin-producing Escherichia coli infection</t>
+        </is>
+      </c>
+      <c r="J402" t="inlineStr">
+        <is>
+          <t>产志贺毒素大肠杆菌感染</t>
+        </is>
+      </c>
+      <c r="K402" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L402" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M402" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N402" t="n">
+        <v>984</v>
+      </c>
+      <c r="O402" t="n">
+        <v>984</v>
+      </c>
+      <c r="R402" t="n">
+        <v>10.79708136456674</v>
+      </c>
+      <c r="S402" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U402" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_STEC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA402" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO402" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP402" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ402" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS402" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_STEC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT402" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU402" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV402" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW402" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX402" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY402" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ402" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA402" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB402" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC402" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>D115</t>
+        </is>
+      </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>Shiga toxin-producing Escherichia coli infection</t>
+        </is>
+      </c>
+      <c r="J403" t="inlineStr">
+        <is>
+          <t>产志贺毒素大肠杆菌感染</t>
+        </is>
+      </c>
+      <c r="K403" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L403" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M403" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N403" t="n">
+        <v>984</v>
+      </c>
+      <c r="O403" t="n">
+        <v>984</v>
+      </c>
+      <c r="U403" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_STEC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V403" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_STEC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W403" t="inlineStr">
+        <is>
+          <t>SRC_AT_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X403" t="inlineStr">
+        <is>
+          <t>STEC/VTEC infection</t>
+        </is>
+      </c>
+      <c r="Y403" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z403" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA403" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB403" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC403" t="inlineStr">
+        <is>
+          <t>country:AT:national</t>
+        </is>
+      </c>
+      <c r="AD403" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE403" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF403" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG403" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH403" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI403" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ403" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK403" t="inlineStr">
+        <is>
+          <t>Austria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM403" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN403" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO403" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP403" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ403" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS403" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_STEC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT403" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU403" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV403" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW403" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX403" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY403" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ403" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA403" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB403" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC403" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>D122</t>
+        </is>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>Trichinellosis</t>
+        </is>
+      </c>
+      <c r="J404" t="inlineStr">
+        <is>
+          <t>旋毛虫病</t>
+        </is>
+      </c>
+      <c r="K404" t="inlineStr">
+        <is>
+          <t>Parasitic</t>
+        </is>
+      </c>
+      <c r="L404" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M404" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N404" t="n">
+        <v>1</v>
+      </c>
+      <c r="O404" t="n">
+        <v>1</v>
+      </c>
+      <c r="R404" t="n">
+        <v>0.01097264366317758</v>
+      </c>
+      <c r="S404" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U404" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_TRIC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA404" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO404" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP404" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ404" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS404" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_TRIC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT404" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU404" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV404" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW404" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX404" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY404" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ404" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA404" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB404" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC404" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>D122</t>
+        </is>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>Trichinellosis</t>
+        </is>
+      </c>
+      <c r="J405" t="inlineStr">
+        <is>
+          <t>旋毛虫病</t>
+        </is>
+      </c>
+      <c r="K405" t="inlineStr">
+        <is>
+          <t>Parasitic</t>
+        </is>
+      </c>
+      <c r="L405" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="M405" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="N405" t="n">
+        <v>1</v>
+      </c>
+      <c r="O405" t="n">
+        <v>1</v>
+      </c>
+      <c r="U405" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_TRIC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V405" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_TRIC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W405" t="inlineStr">
+        <is>
+          <t>SRC_AT_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X405" t="inlineStr">
+        <is>
+          <t>Trichinellosis</t>
+        </is>
+      </c>
+      <c r="Y405" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z405" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA405" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB405" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC405" t="inlineStr">
+        <is>
+          <t>country:AT:national</t>
+        </is>
+      </c>
+      <c r="AD405" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE405" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF405" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG405" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH405" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI405" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ405" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK405" t="inlineStr">
+        <is>
+          <t>Austria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM405" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN405" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO405" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP405" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ405" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS405" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_TRIC_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT405" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU405" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV405" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW405" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX405" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY405" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ405" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA405" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB405" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC405" t="inlineStr">
         <is>
           <t>official_monthly_csv</t>
         </is>
@@ -76658,7 +80195,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>193</v>
+        <v>202</v>
       </c>
     </row>
     <row r="10">
@@ -76668,7 +80205,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>386</v>
+        <v>404</v>
       </c>
     </row>
     <row r="11">
@@ -76688,7 +80225,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>193</v>
+        <v>202</v>
       </c>
     </row>
     <row r="13">
@@ -76720,7 +80257,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>75394</v>
+        <v>85491</v>
       </c>
     </row>
     <row r="16">

</xml_diff>